<commit_message>
Latest generated outputs 2026-10-22
</commit_message>
<xml_diff>
--- a/generated/spreadsheet/lawful-development-certficate-proposed-work-to-a-listed-building-ldc-proposed-work-lb.xlsx
+++ b/generated/spreadsheet/lawful-development-certficate-proposed-work-to-a-listed-building-ldc-proposed-work-lb.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I91"/>
+  <dimension ref="A1:I92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="72" customWidth="1" min="1" max="1"/>
@@ -2836,7 +2836,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Listed building grade</t>
+          <t>Listed building grade known</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr"/>
@@ -2844,12 +2844,12 @@
       <c r="F69" s="2" t="inlineStr"/>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>The grade of the listed building, selected from the listed-building-grade codelist or "don't know"</t>
+          <t>Set to true if the applicant knows the listed building grade. Set to false if they do not know it.</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
@@ -2863,7 +2863,7 @@
       <c r="B70" s="2" t="n"/>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Listed building</t>
+          <t>Listed building grade</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr"/>
@@ -2871,17 +2871,17 @@
       <c r="F70" s="2" t="inlineStr"/>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Listed building reference for cross-referencing with listed building records</t>
+          <t>The grade of the listed building, selected from the listed-building-grade codelist</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -2890,7 +2890,7 @@
       <c r="B71" s="2" t="n"/>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Provided by</t>
+          <t>Listed building</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr"/>
@@ -2898,12 +2898,12 @@
       <c r="F71" s="2" t="inlineStr"/>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Source of the listed building grade information</t>
+          <t>Listed building reference for cross-referencing with listed building records</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
@@ -2913,19 +2913,11 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>Pre-application advice</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>Details of pre-application advice previously received from the planning authority</t>
-        </is>
-      </c>
+      <c r="A72" s="2" t="n"/>
+      <c r="B72" s="2" t="n"/>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Pre-application advice sought</t>
+          <t>Provided by</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr"/>
@@ -2933,26 +2925,34 @@
       <c r="F72" s="2" t="inlineStr"/>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Whether pre-application advice has been sought from the planning authority</t>
+          <t>Source of the listed building grade information</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n"/>
-      <c r="B73" s="2" t="n"/>
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Pre-application advice</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Details of pre-application advice previously received from the planning authority</t>
+        </is>
+      </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Planning officer name</t>
+          <t>Pre-application advice sought</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr"/>
@@ -2960,17 +2960,17 @@
       <c r="F73" s="2" t="inlineStr"/>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Name of the planning officer who provided the pre-application advice</t>
+          <t>Whether pre-application advice has been sought from the planning authority</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       <c r="B74" s="2" t="n"/>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Planning officer name</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr"/>
@@ -2987,7 +2987,7 @@
       <c r="F74" s="2" t="inlineStr"/>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>A unique reference for the data item</t>
+          <t>Name of the planning officer who provided the pre-application advice</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -3006,7 +3006,7 @@
       <c r="B75" s="2" t="n"/>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Advice date</t>
+          <t>Reference</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr"/>
@@ -3014,12 +3014,12 @@
       <c r="F75" s="2" t="inlineStr"/>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Date when pre-application advice was received, in YYYY-MM-DD format</t>
+          <t>A unique reference for the data item</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
@@ -3033,7 +3033,7 @@
       <c r="B76" s="2" t="n"/>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Advice summary</t>
+          <t>Advice date</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr"/>
@@ -3041,12 +3041,12 @@
       <c r="F76" s="2" t="inlineStr"/>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Summary of the pre-application advice received from the planning authority</t>
+          <t>Date when pre-application advice was received, in YYYY-MM-DD format</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
@@ -3056,47 +3056,43 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>Site details</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>Where the proposed development will be built.</t>
-        </is>
-      </c>
+      <c r="A77" s="2" t="n"/>
+      <c r="B77" s="2" t="n"/>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Site locations[]</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
-        <is>
-          <t>Site boundary</t>
-        </is>
-      </c>
+          <t>Advice summary</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr"/>
       <c r="E77" s="2" t="inlineStr"/>
       <c r="F77" s="2" t="inlineStr"/>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>A polygon or multipolygon boundary</t>
+          <t>Summary of the pre-application advice received from the planning authority</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>multipolygon</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n"/>
-      <c r="B78" s="2" t="n"/>
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Site details</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Where the proposed development will be built.</t>
+        </is>
+      </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
           <t>Site locations[]</t>
@@ -3104,23 +3100,19 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Site address</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>Address Text</t>
-        </is>
-      </c>
+          <t>Site boundary</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr"/>
       <c r="F78" s="2" t="inlineStr"/>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Text representation of an address or site</t>
+          <t>A polygon or multipolygon boundary</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>multipolygon</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
@@ -3144,13 +3136,13 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Postcode</t>
+          <t>Address Text</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr"/>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Postcode for a contact address or site</t>
+          <t>Text representation of an address or site</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -3160,7 +3152,7 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -3179,13 +3171,13 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>UPRNs[]</t>
+          <t>Postcode</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr"/>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Unique Property Reference Numbers (UPRNs) for existing premises within a site boundary</t>
+          <t>Postcode for a contact address or site</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -3214,13 +3206,13 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>USRNs[]</t>
+          <t>UPRNs[]</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr"/>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Unique Street Reference Numbers (USRNs) associated with the site</t>
+          <t>Unique Property Reference Numbers (UPRNs) for existing premises within a site boundary</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
@@ -3244,19 +3236,23 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Easting</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr"/>
+          <t>Site address</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>USRNs[]</t>
+        </is>
+      </c>
       <c r="F82" s="2" t="inlineStr"/>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Easting coordinate in British National Grid (EPSG:27700)</t>
+          <t>Unique Street Reference Numbers (USRNs) associated with the site</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
@@ -3275,14 +3271,14 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Northing</t>
+          <t>Easting</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr"/>
       <c r="F83" s="2" t="inlineStr"/>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Northing coordinate in British National Grid (EPSG:27700)</t>
+          <t>Easting coordinate in British National Grid (EPSG:27700)</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -3306,19 +3302,19 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Latitude</t>
+          <t>Northing</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr"/>
       <c r="F84" s="2" t="inlineStr"/>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Latitude coordinate in WGS84 (EPSG:4326)</t>
+          <t>Northing coordinate in British National Grid (EPSG:27700)</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>latitude</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
@@ -3337,19 +3333,19 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Longitude</t>
+          <t>Latitude</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr"/>
       <c r="F85" s="2" t="inlineStr"/>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Longitude coordinate in WGS84 (EPSG:4326)</t>
+          <t>Latitude coordinate in WGS84 (EPSG:4326)</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>longitude</t>
+          <t>latitude</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr">
@@ -3359,46 +3355,50 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="inlineStr">
-        <is>
-          <t>Site Visit Details</t>
-        </is>
-      </c>
-      <c r="B86" s="2" t="inlineStr">
-        <is>
-          <t>Information to help the planning authority arrange a site visit</t>
-        </is>
-      </c>
+      <c r="A86" s="2" t="n"/>
+      <c r="B86" s="2" t="n"/>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Site seen from public area</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="inlineStr"/>
+          <t>Site locations[]</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Longitude</t>
+        </is>
+      </c>
       <c r="E86" s="2" t="inlineStr"/>
       <c r="F86" s="2" t="inlineStr"/>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Can site be seen from a public road, public footpath, bridleway or other public land</t>
+          <t>Longitude coordinate in WGS84 (EPSG:4326)</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>longitude</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n"/>
-      <c r="B87" s="2" t="n"/>
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Site Visit Details</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Information to help the planning authority arrange a site visit</t>
+        </is>
+      </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Site visit contact type</t>
+          <t>Site seen from public area</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr"/>
@@ -3406,12 +3406,12 @@
       <c r="F87" s="2" t="inlineStr"/>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Indicates who the authority should contact to arrange a site visit</t>
+          <t>Can site be seen from a public road, public footpath, bridleway or other public land</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr">
@@ -3425,7 +3425,7 @@
       <c r="B88" s="2" t="n"/>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Contact reference</t>
+          <t>Site visit contact type</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr"/>
@@ -3433,17 +3433,17 @@
       <c r="F88" s="2" t="inlineStr"/>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>The reference of the applicant or agent who should be contacted for site visits</t>
+          <t>Indicates who the authority should contact to arrange a site visit</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -3452,19 +3452,15 @@
       <c r="B89" s="2" t="n"/>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Other site visit contact</t>
-        </is>
-      </c>
-      <c r="D89" s="2" t="inlineStr">
-        <is>
-          <t>Full name</t>
-        </is>
-      </c>
+          <t>Contact reference</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr"/>
       <c r="E89" s="2" t="inlineStr"/>
       <c r="F89" s="2" t="inlineStr"/>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>The complete name of a person</t>
+          <t>The reference of the applicant or agent who should be contacted for site visits</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
@@ -3474,7 +3470,7 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -3488,14 +3484,14 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Phone number</t>
+          <t>Full name</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr"/>
       <c r="F90" s="2" t="inlineStr"/>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>A phone number</t>
+          <t>The complete name of a person</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
@@ -3519,22 +3515,53 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Phone number</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr"/>
       <c r="F91" s="2" t="inlineStr"/>
       <c r="G91" s="2" t="inlineStr">
         <is>
+          <t>A phone number</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n"/>
+      <c r="B92" s="2" t="n"/>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Other site visit contact</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="inlineStr"/>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
           <t>The email address that can be used for electronic correspondence with the individual</t>
         </is>
       </c>
-      <c r="H91" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="I91" s="2" t="inlineStr">
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
@@ -3544,34 +3571,34 @@
   <mergeCells count="30">
     <mergeCell ref="B49"/>
     <mergeCell ref="A37:A43"/>
+    <mergeCell ref="B78:B86"/>
     <mergeCell ref="A2:A19"/>
+    <mergeCell ref="A69:A72"/>
     <mergeCell ref="A50:A51"/>
-    <mergeCell ref="A72:A76"/>
     <mergeCell ref="A44"/>
     <mergeCell ref="B37:B43"/>
     <mergeCell ref="B45"/>
     <mergeCell ref="B52:B68"/>
-    <mergeCell ref="B86:B91"/>
+    <mergeCell ref="A87:A92"/>
     <mergeCell ref="A49"/>
     <mergeCell ref="B24:B32"/>
     <mergeCell ref="A33:A36"/>
-    <mergeCell ref="B72:B76"/>
+    <mergeCell ref="A73:A77"/>
     <mergeCell ref="A45"/>
-    <mergeCell ref="A86:A91"/>
+    <mergeCell ref="B69:B72"/>
+    <mergeCell ref="B87:B92"/>
     <mergeCell ref="A20:A23"/>
-    <mergeCell ref="A69:A71"/>
-    <mergeCell ref="A77:A85"/>
     <mergeCell ref="B46:B48"/>
     <mergeCell ref="B33:B36"/>
     <mergeCell ref="A24:A32"/>
     <mergeCell ref="B44"/>
     <mergeCell ref="B20:B23"/>
+    <mergeCell ref="A78:A86"/>
+    <mergeCell ref="B73:B77"/>
     <mergeCell ref="A52:A68"/>
     <mergeCell ref="B2:B19"/>
     <mergeCell ref="A46:A48"/>
-    <mergeCell ref="B69:B71"/>
     <mergeCell ref="B50:B51"/>
-    <mergeCell ref="B77:B85"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>